<commit_message>
Add SOH report for 2026-10-01
</commit_message>
<xml_diff>
--- a/reports/SOH_30_09_2026.xlsx
+++ b/reports/SOH_30_09_2026.xlsx
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>21000</v>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>1</v>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>603</v>
+        <v>599</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>8000</v>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>828</v>
+        <v>827</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>25000</v>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>40000</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1150</v>
+        <v>1130</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>-23</v>
+        <v>-30</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>40000</v>
@@ -1469,7 +1469,7 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>48000</v>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="E44" s="3" t="n">
         <v>4500</v>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="E45" s="3" t="n">
         <v>12500</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>632</v>
+        <v>614</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>51000</v>
@@ -2169,7 +2169,7 @@
         </is>
       </c>
       <c r="D62" s="2" t="n">
-        <v>921</v>
+        <v>906</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>51000</v>
@@ -2533,7 +2533,7 @@
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E75" s="3" t="n">
         <v>4000</v>
@@ -2561,7 +2561,7 @@
         </is>
       </c>
       <c r="D76" s="2" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>4000</v>
@@ -3429,7 +3429,7 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E107" s="3" t="n">
         <v>1</v>
@@ -3485,7 +3485,7 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>2838</v>
+        <v>2837</v>
       </c>
       <c r="E109" s="3" t="n">
         <v>3876</v>
@@ -3513,7 +3513,7 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>2642</v>
+        <v>2641</v>
       </c>
       <c r="E110" s="3" t="n">
         <v>3500</v>
@@ -4769,7 +4769,7 @@
         </is>
       </c>
       <c r="D155" s="2" t="n">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E155" s="3" t="n">
         <v>1</v>
@@ -4881,7 +4881,7 @@
         </is>
       </c>
       <c r="D159" s="2" t="n">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="E159" s="3" t="n">
         <v>1</v>
@@ -5365,7 +5365,7 @@
         </is>
       </c>
       <c r="D177" s="2" t="n">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E177" s="3" t="n">
         <v>1</v>
@@ -6177,7 +6177,7 @@
         </is>
       </c>
       <c r="D207" s="2" t="n">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E207" s="3" t="n">
         <v>1</v>
@@ -6685,7 +6685,7 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="E226" s="3" t="n">
         <v>1</v>
@@ -10749,7 +10749,7 @@
         <v>73</v>
       </c>
       <c r="E372" s="3" t="n">
-        <v>0</v>
+        <v>39772</v>
       </c>
       <c r="F372" t="inlineStr">
         <is>
@@ -11866,7 +11866,7 @@
         </is>
       </c>
       <c r="D412" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E412" s="3" t="n">
         <v>53004</v>
@@ -13294,7 +13294,7 @@
         </is>
       </c>
       <c r="D463" s="2" t="n">
-        <v>151</v>
+        <v>126</v>
       </c>
       <c r="E463" s="3" t="n">
         <v>6441</v>
@@ -15450,7 +15450,7 @@
         </is>
       </c>
       <c r="D540" s="2" t="n">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="E540" s="3" t="n">
         <v>7573</v>
@@ -20379,7 +20379,7 @@
         </is>
       </c>
       <c r="D716" s="2" t="n">
-        <v>486</v>
+        <v>474</v>
       </c>
       <c r="E716" s="3" t="n">
         <v>5340</v>
@@ -23067,7 +23067,7 @@
         </is>
       </c>
       <c r="D812" s="2" t="n">
-        <v>355</v>
+        <v>343</v>
       </c>
       <c r="E812" s="3" t="n">
         <v>5764</v>
@@ -23600,7 +23600,7 @@
         </is>
       </c>
       <c r="D831" s="2" t="n">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="E831" s="3" t="n">
         <v>3052</v>
@@ -28756,7 +28756,7 @@
         </is>
       </c>
       <c r="D1015" s="2" t="n">
-        <v>733</v>
+        <v>709</v>
       </c>
       <c r="E1015" s="3" t="n">
         <v>2930</v>
@@ -29681,7 +29681,7 @@
         </is>
       </c>
       <c r="D1048" s="2" t="n">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="E1048" s="3" t="n">
         <v>6142</v>
@@ -30129,7 +30129,7 @@
         </is>
       </c>
       <c r="D1064" s="2" t="n">
-        <v>593</v>
+        <v>581</v>
       </c>
       <c r="E1064" s="3" t="n">
         <v>3247</v>
@@ -30297,7 +30297,7 @@
         </is>
       </c>
       <c r="D1070" s="2" t="n">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="E1070" s="3" t="n">
         <v>18503</v>
@@ -30325,7 +30325,7 @@
         </is>
       </c>
       <c r="D1071" s="2" t="n">
-        <v>322</v>
+        <v>302</v>
       </c>
       <c r="E1071" s="3" t="n">
         <v>10760</v>
@@ -30437,7 +30437,7 @@
         </is>
       </c>
       <c r="D1075" s="2" t="n">
-        <v>562</v>
+        <v>550</v>
       </c>
       <c r="E1075" s="3" t="n">
         <v>9226</v>
@@ -32705,7 +32705,7 @@
         </is>
       </c>
       <c r="D1156" s="2" t="n">
-        <v>528</v>
+        <v>516</v>
       </c>
       <c r="E1156" s="3" t="n">
         <v>3088</v>
@@ -32761,7 +32761,7 @@
         </is>
       </c>
       <c r="D1158" s="2" t="n">
-        <v>369</v>
+        <v>345</v>
       </c>
       <c r="E1158" s="3" t="n">
         <v>9174</v>
@@ -37325,7 +37325,7 @@
         </is>
       </c>
       <c r="D1321" s="2" t="n">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="E1321" s="3" t="n">
         <v>5674</v>
@@ -38529,7 +38529,7 @@
         </is>
       </c>
       <c r="D1364" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E1364" s="3" t="n">
         <v>18059</v>
@@ -38585,7 +38585,7 @@
         </is>
       </c>
       <c r="D1366" s="2" t="n">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="E1366" s="3" t="n">
         <v>10847</v>
@@ -40349,7 +40349,7 @@
         </is>
       </c>
       <c r="D1429" s="2" t="n">
-        <v>790</v>
+        <v>778</v>
       </c>
       <c r="E1429" s="3" t="n">
         <v>3140</v>

</xml_diff>